<commit_message>
Add batch summary workbook generation and error handling in CLI
Implement a new function to write a batch summary workbook after processing multiple DEMs, enhancing output reporting capabilities. Update the main configuration flow to conditionally generate the summary workbook based on the number of batch jobs processed. Introduce error handling for workbook writing operations to ensure robustness. Additionally, add tests to validate the new functionality and confirm the correctness of the generated Excel files.
</commit_message>
<xml_diff>
--- a/sonuclar_out_/synth_plane_16384x16384_dx0.05_seed0_20260315_213848/results.xlsx
+++ b/sonuclar_out_/synth_plane_16384x16384_dx0.05_seed0_20260315_213848/results.xlsx
@@ -1797,8 +1797,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="RunInfoTable" displayName="RunInfoTable" ref="A1:B53" headerRowCount="1">
-  <autoFilter ref="A1:B53"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="RunInfoTable" displayName="RunInfoTable" ref="A1:B55" headerRowCount="1">
+  <autoFilter ref="A1:B55"/>
   <tableColumns count="2">
     <tableColumn id="1" name="key"/>
     <tableColumn id="2" name="value"/>
@@ -2299,7 +2299,7 @@
         <v>268369924</v>
       </c>
       <c r="I2" t="n">
-        <v>7.682050698262174</v>
+        <v>5.650267199496739</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
@@ -2356,7 +2356,7 @@
         <v>268369924</v>
       </c>
       <c r="I3" t="n">
-        <v>65.78858370281523</v>
+        <v>57.18830979574705</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
@@ -2413,7 +2413,7 @@
         <v>268369924</v>
       </c>
       <c r="I4" t="n">
-        <v>2081.548187398526</v>
+        <v>2184.058027800347</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
@@ -2476,7 +2476,7 @@
         <v>268369924</v>
       </c>
       <c r="I5" t="n">
-        <v>15.69642789848149</v>
+        <v>14.46445210085949</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -2575,7 +2575,7 @@
         <v>670761</v>
       </c>
       <c r="F7" t="n">
-        <v>865394.9605927564</v>
+        <v>865394.9605927563</v>
       </c>
       <c r="G7" t="n">
         <v>1.290168868781513</v>
@@ -2584,10 +2584,10 @@
         <v>67076100</v>
       </c>
       <c r="I7" t="n">
-        <v>2.076502800628077</v>
+        <v>1.50725369999418</v>
       </c>
       <c r="J7" t="n">
-        <v>5.627892700023949</v>
+        <v>5.809013100049924</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -2631,10 +2631,10 @@
         <v>67076100</v>
       </c>
       <c r="I8" t="n">
-        <v>16.38930120074656</v>
+        <v>14.76537529908819</v>
       </c>
       <c r="J8" t="n">
-        <v>5.627892700023949</v>
+        <v>5.809013100049924</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -2678,10 +2678,10 @@
         <v>67076100</v>
       </c>
       <c r="I9" t="n">
-        <v>546.0752359002945</v>
+        <v>547.2294839996612</v>
       </c>
       <c r="J9" t="n">
-        <v>5.627892700023949</v>
+        <v>5.809013100049924</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -2731,10 +2731,10 @@
         <v>67076100</v>
       </c>
       <c r="I10" t="n">
-        <v>4.142207900993526</v>
+        <v>3.529107398819178</v>
       </c>
       <c r="J10" t="n">
-        <v>5.627892700023949</v>
+        <v>5.809013100049924</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -2778,10 +2778,10 @@
         <v>2676496</v>
       </c>
       <c r="I11" t="n">
-        <v>0.07275269983801991</v>
+        <v>0.06602799985557795</v>
       </c>
       <c r="J11" t="n">
-        <v>3.403379699971993</v>
+        <v>3.609141600027215</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -2825,10 +2825,10 @@
         <v>2676496</v>
       </c>
       <c r="I12" t="n">
-        <v>0.4674302999046631</v>
+        <v>0.5712813001009636</v>
       </c>
       <c r="J12" t="n">
-        <v>3.403379699971993</v>
+        <v>3.609141600027215</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
@@ -2863,7 +2863,7 @@
         <v>669124</v>
       </c>
       <c r="F13" t="n">
-        <v>824441.9861349808</v>
+        <v>824441.9861349809</v>
       </c>
       <c r="G13" t="n">
         <v>1.232121379796541</v>
@@ -2872,10 +2872,10 @@
         <v>2676496</v>
       </c>
       <c r="I13" t="n">
-        <v>20.41015920002246</v>
+        <v>37.99743129994022</v>
       </c>
       <c r="J13" t="n">
-        <v>3.403379699971993</v>
+        <v>3.609141600027215</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
@@ -2925,10 +2925,10 @@
         <v>2676496</v>
       </c>
       <c r="I14" t="n">
-        <v>0.1374688994837925</v>
+        <v>0.1160655996645801</v>
       </c>
       <c r="J14" t="n">
-        <v>3.403379699971993</v>
+        <v>3.609141600027215</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
@@ -2963,7 +2963,7 @@
         <v>667489</v>
       </c>
       <c r="F15" t="n">
-        <v>749354.3278026374</v>
+        <v>749354.3278026375</v>
       </c>
       <c r="G15" t="n">
         <v>1.122646706990883</v>
@@ -2972,10 +2972,10 @@
         <v>667489</v>
       </c>
       <c r="I15" t="n">
-        <v>0.01495390007039532</v>
+        <v>0.01322989992331713</v>
       </c>
       <c r="J15" t="n">
-        <v>3.405729599995539</v>
+        <v>3.551354300056119</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
@@ -3019,10 +3019,10 @@
         <v>667489</v>
       </c>
       <c r="I16" t="n">
-        <v>0.09982170007424429</v>
+        <v>0.0977692999294959</v>
       </c>
       <c r="J16" t="n">
-        <v>3.405729599995539</v>
+        <v>3.551354300056119</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
@@ -3057,7 +3057,7 @@
         <v>667489</v>
       </c>
       <c r="F17" t="n">
-        <v>755910.4055846768</v>
+        <v>755910.4055846769</v>
       </c>
       <c r="G17" t="n">
         <v>1.132468708225419</v>
@@ -3066,10 +3066,10 @@
         <v>667489</v>
       </c>
       <c r="I17" t="n">
-        <v>6.364683800027706</v>
+        <v>7.881803599884734</v>
       </c>
       <c r="J17" t="n">
-        <v>3.405729599995539</v>
+        <v>3.551354300056119</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -3110,7 +3110,7 @@
         <v>667489</v>
       </c>
       <c r="F18" t="n">
-        <v>756036.7141654211</v>
+        <v>756036.7141654212</v>
       </c>
       <c r="G18" t="n">
         <v>1.132657937682001</v>
@@ -3119,10 +3119,10 @@
         <v>667489</v>
       </c>
       <c r="I18" t="n">
-        <v>0.04436070012161508</v>
+        <v>0.02684159995988011</v>
       </c>
       <c r="J18" t="n">
-        <v>3.405729599995539</v>
+        <v>3.551354300056119</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
@@ -3166,10 +3166,10 @@
         <v>166464</v>
       </c>
       <c r="I19" t="n">
-        <v>0.002922300016507506</v>
+        <v>0.002858000108972192</v>
       </c>
       <c r="J19" t="n">
-        <v>3.382380300026853</v>
+        <v>3.528990099963266</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
@@ -3204,7 +3204,7 @@
         <v>665856</v>
       </c>
       <c r="F20" t="n">
-        <v>719919.150540015</v>
+        <v>719919.1505400151</v>
       </c>
       <c r="G20" t="n">
         <v>1.0811934570538</v>
@@ -3213,10 +3213,10 @@
         <v>166464</v>
       </c>
       <c r="I20" t="n">
-        <v>0.01857339992420748</v>
+        <v>0.02241650002542883</v>
       </c>
       <c r="J20" t="n">
-        <v>3.382380300026853</v>
+        <v>3.528990099963266</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
@@ -3260,10 +3260,10 @@
         <v>166464</v>
       </c>
       <c r="I21" t="n">
-        <v>0.7491928999661468</v>
+        <v>1.045753700018395</v>
       </c>
       <c r="J21" t="n">
-        <v>3.382380300026853</v>
+        <v>3.528990099963266</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
@@ -3313,10 +3313,10 @@
         <v>166464</v>
       </c>
       <c r="I22" t="n">
-        <v>0.005460299958940595</v>
+        <v>0.00546890014084056</v>
       </c>
       <c r="J22" t="n">
-        <v>3.382380300026853</v>
+        <v>3.528990099963266</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
@@ -3360,10 +3360,10 @@
         <v>26244</v>
       </c>
       <c r="I23" t="n">
-        <v>0.0002757999463938177</v>
+        <v>0.0003978000022470951</v>
       </c>
       <c r="J23" t="n">
-        <v>3.487434400012717</v>
+        <v>3.630758900020737</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
@@ -3407,10 +3407,10 @@
         <v>26244</v>
       </c>
       <c r="I24" t="n">
-        <v>0.003182000014930964</v>
+        <v>0.003449000010732561</v>
       </c>
       <c r="J24" t="n">
-        <v>3.487434400012717</v>
+        <v>3.630758900020737</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
@@ -3454,10 +3454,10 @@
         <v>26244</v>
       </c>
       <c r="I25" t="n">
-        <v>0.0792984000290744</v>
+        <v>0.08727009996073321</v>
       </c>
       <c r="J25" t="n">
-        <v>3.487434400012717</v>
+        <v>3.630758900020737</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
@@ -3507,10 +3507,10 @@
         <v>26244</v>
       </c>
       <c r="I26" t="n">
-        <v>0.0008853999897837639</v>
+        <v>0.000860599975567311</v>
       </c>
       <c r="J26" t="n">
-        <v>3.487434400012717</v>
+        <v>3.630758900020737</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
@@ -3554,10 +3554,10 @@
         <v>6400</v>
       </c>
       <c r="I27" t="n">
-        <v>0.000133700028527528</v>
+        <v>0.0001548000145703554</v>
       </c>
       <c r="J27" t="n">
-        <v>3.567525999969803</v>
+        <v>3.760430499969516</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
@@ -3601,10 +3601,10 @@
         <v>6400</v>
       </c>
       <c r="I28" t="n">
-        <v>0.0007483999943360686</v>
+        <v>0.0009581000194884837</v>
       </c>
       <c r="J28" t="n">
-        <v>3.567525999969803</v>
+        <v>3.760430499969516</v>
       </c>
       <c r="K28" t="inlineStr">
         <is>
@@ -3648,10 +3648,10 @@
         <v>6400</v>
       </c>
       <c r="I29" t="n">
-        <v>0.02118450001580641</v>
+        <v>0.02230569999665022</v>
       </c>
       <c r="J29" t="n">
-        <v>3.567525999969803</v>
+        <v>3.760430499969516</v>
       </c>
       <c r="K29" t="inlineStr">
         <is>
@@ -3701,10 +3701,10 @@
         <v>6400</v>
       </c>
       <c r="I30" t="n">
-        <v>0.000422900018747896</v>
+        <v>0.0003619000199250877</v>
       </c>
       <c r="J30" t="n">
-        <v>3.567525999969803</v>
+        <v>3.760430499969516</v>
       </c>
       <c r="K30" t="inlineStr">
         <is>
@@ -3748,10 +3748,10 @@
         <v>1521</v>
       </c>
       <c r="I31" t="n">
-        <v>6.940000457689166e-05</v>
+        <v>7.449998520314693e-05</v>
       </c>
       <c r="J31" t="n">
-        <v>3.73389649996534</v>
+        <v>3.933846300002187</v>
       </c>
       <c r="K31" t="inlineStr">
         <is>
@@ -3795,10 +3795,10 @@
         <v>1521</v>
       </c>
       <c r="I32" t="n">
-        <v>0.0002442999975755811</v>
+        <v>0.0002716000308282673</v>
       </c>
       <c r="J32" t="n">
-        <v>3.73389649996534</v>
+        <v>3.933846300002187</v>
       </c>
       <c r="K32" t="inlineStr">
         <is>
@@ -3842,10 +3842,10 @@
         <v>1521</v>
       </c>
       <c r="I33" t="n">
-        <v>0.006189999985508621</v>
+        <v>0.006427599990274757</v>
       </c>
       <c r="J33" t="n">
-        <v>3.73389649996534</v>
+        <v>3.933846300002187</v>
       </c>
       <c r="K33" t="inlineStr">
         <is>
@@ -3895,10 +3895,10 @@
         <v>1521</v>
       </c>
       <c r="I34" t="n">
-        <v>0.0001839999458752573</v>
+        <v>0.0002170999650843441</v>
       </c>
       <c r="J34" t="n">
-        <v>3.73389649996534</v>
+        <v>3.933846300002187</v>
       </c>
       <c r="K34" t="inlineStr">
         <is>
@@ -3942,10 +3942,10 @@
         <v>196</v>
       </c>
       <c r="I35" t="n">
-        <v>5.339999916031957e-05</v>
+        <v>0.0001357000437565148</v>
       </c>
       <c r="J35" t="n">
-        <v>5.181329400045797</v>
+        <v>5.324968600005377</v>
       </c>
       <c r="K35" t="inlineStr">
         <is>
@@ -3989,10 +3989,10 @@
         <v>196</v>
       </c>
       <c r="I36" t="n">
-        <v>0.0001169999595731497</v>
+        <v>0.0001211999915540218</v>
       </c>
       <c r="J36" t="n">
-        <v>5.181329400045797</v>
+        <v>5.324968600005377</v>
       </c>
       <c r="K36" t="inlineStr">
         <is>
@@ -4036,10 +4036,10 @@
         <v>196</v>
       </c>
       <c r="I37" t="n">
-        <v>0.002391399990301579</v>
+        <v>0.002684999955818057</v>
       </c>
       <c r="J37" t="n">
-        <v>5.181329400045797</v>
+        <v>5.324968600005377</v>
       </c>
       <c r="K37" t="inlineStr">
         <is>
@@ -4089,10 +4089,10 @@
         <v>196</v>
       </c>
       <c r="I38" t="n">
-        <v>0.0001466000103391707</v>
+        <v>0.0001795999705791473</v>
       </c>
       <c r="J38" t="n">
-        <v>5.181329400045797</v>
+        <v>5.324968600005377</v>
       </c>
       <c r="K38" t="inlineStr">
         <is>
@@ -4174,7 +4174,7 @@
         <v>0.1</v>
       </c>
       <c r="B3" t="n">
-        <v>865394.9605927564</v>
+        <v>865394.9605927563</v>
       </c>
       <c r="C3" t="n">
         <v>866603.4905840222</v>
@@ -4197,7 +4197,7 @@
         <v>844716.5965149167</v>
       </c>
       <c r="D4" t="n">
-        <v>824441.9861349808</v>
+        <v>824441.9861349809</v>
       </c>
       <c r="E4" t="n">
         <v>825491.5320733978</v>
@@ -4208,16 +4208,16 @@
         <v>1</v>
       </c>
       <c r="B5" t="n">
-        <v>749354.3278026374</v>
+        <v>749354.3278026375</v>
       </c>
       <c r="C5" t="n">
         <v>797082.4788724037</v>
       </c>
       <c r="D5" t="n">
-        <v>755910.4055846768</v>
+        <v>755910.4055846769</v>
       </c>
       <c r="E5" t="n">
-        <v>756036.7141654211</v>
+        <v>756036.7141654212</v>
       </c>
     </row>
     <row r="6">
@@ -4228,7 +4228,7 @@
         <v>686613.3653028569</v>
       </c>
       <c r="C6" t="n">
-        <v>719919.150540015</v>
+        <v>719919.1505400151</v>
       </c>
       <c r="D6" t="n">
         <v>691007.5050956833</v>
@@ -4408,7 +4408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B53"/>
+  <dimension ref="A1:B55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4431,7 +4431,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-03-17T08:11:14.494246+00:00</t>
+          <t>2026-03-17T09:20:38.634283+00:00</t>
         </is>
       </c>
     </row>
@@ -4664,316 +4664,338 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>versions.rasterio</t>
+          <t>versions.numba</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>1.5.0</t>
+          <t>0.64.0</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>versions.scipy</t>
+          <t>versions.rasterio</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>1.17.1</t>
+          <t>1.5.0</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>versions.pandas</t>
+          <t>versions.scipy</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>3.0.1</t>
+          <t>1.17.1</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>versions.matplotlib</t>
+          <t>versions.pandas</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>3.10.8</t>
+          <t>3.0.1</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>params.gsd_specs</t>
+          <t>versions.matplotlib</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>["native", "0.1", "0.5", "1", "2", "5", "10", "20", "50"]</t>
+          <t>3.10.8</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>params.gsd_list</t>
+          <t>params.gsd_specs</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>[0.05, 0.1, 0.5, 1.0, 2.0, 5.0, 10.0, 20.0, 50.0]</t>
+          <t>["native", "0.1", "0.5", "1", "2", "5", "10", "20", "50"]</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>params.methods</t>
+          <t>params.gsd_list</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>["jenness_window_8tri", "sector_adaptive_jenness_integral", "tin_2tri_cell", "gradient_multiplier"]</t>
+          <t>[0.05, 0.1, 0.5, 1.0, 2.0, 5.0, 10.0, 20.0, 50.0]</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>params.resampling</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>bilinear</t>
-        </is>
+          <t>params.allow_upsample</t>
+        </is>
+      </c>
+      <c r="B31" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>params.nodata_override</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr"/>
+          <t>params.methods</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>["jenness_window_8tri", "sector_adaptive_jenness_integral", "tin_2tri_cell", "gradient_multiplier"]</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>params.slope_method</t>
+          <t>params.resampling</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>horn</t>
+          <t>bilinear</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>params.jenness_weight</t>
-        </is>
-      </c>
-      <c r="B34" t="n">
-        <v>0.25</v>
-      </c>
+          <t>params.nodata_override</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>params.integral_N</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>5</v>
+          <t>params.slope_method</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>horn</t>
+        </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>params.adaptive_rel_tol</t>
+          <t>params.jenness_weight</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>0.0001</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>params.adaptive_abs_tol</t>
+          <t>params.integral_N</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>params.adaptive_max_level</t>
+          <t>params.adaptive_rel_tol</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>5</v>
+        <v>0.0001</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>params.adaptive_min_N</t>
+          <t>params.adaptive_abs_tol</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>params.adaptive_roughness_fastpath</t>
-        </is>
-      </c>
-      <c r="B40" t="b">
-        <v>1</v>
+          <t>params.adaptive_max_level</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>params.adaptive_roughness_threshold</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr"/>
+          <t>params.adaptive_min_N</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>params.sector_jenness_rel_tol</t>
-        </is>
-      </c>
-      <c r="B42" t="n">
-        <v>0.0001</v>
+          <t>params.adaptive_roughness_fastpath</t>
+        </is>
+      </c>
+      <c r="B42" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>params.sector_jenness_abs_tol</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>0</v>
-      </c>
+          <t>params.adaptive_roughness_threshold</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>params.sector_jenness_max_level</t>
+          <t>params.sector_jenness_rel_tol</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>5</v>
+        <v>0.0001</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>params.sector_jenness_min_samples</t>
+          <t>params.sector_jenness_abs_tol</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>params.sigma_mode</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>mult</t>
-        </is>
+          <t>params.sector_jenness_max_level</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>params.sigma_m_values</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>[2.0, 5.0]</t>
-        </is>
+          <t>params.sector_jenness_min_samples</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>params.roi</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr"/>
+          <t>params.sigma_mode</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>mult</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>params.roi_id_field</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr"/>
+          <t>params.sigma_m_values</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>[2.0, 5.0]</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>params.roi_mode</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>mask</t>
-        </is>
-      </c>
+          <t>params.roi</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>params.roi_all_touched</t>
-        </is>
-      </c>
-      <c r="B51" t="b">
-        <v>0</v>
-      </c>
+          <t>params.roi_id_field</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>params.roi_only</t>
-        </is>
-      </c>
-      <c r="B52" t="b">
-        <v>0</v>
+          <t>params.roi_mode</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>mask</t>
+        </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
+          <t>params.roi_all_touched</t>
+        </is>
+      </c>
+      <c r="B53" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>params.roi_only</t>
+        </is>
+      </c>
+      <c r="B54" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
           <t>params.workers</t>
         </is>
       </c>
-      <c r="B53" t="n">
+      <c r="B55" t="n">
         <v>8</v>
       </c>
     </row>
@@ -5106,7 +5128,7 @@
         <v>0.1</v>
       </c>
       <c r="B130" s="7" t="n">
-        <v>865394.9605927564</v>
+        <v>865394.9605927563</v>
       </c>
       <c r="C130" s="7" t="n">
         <v>866603.4905840222</v>
@@ -5130,7 +5152,7 @@
         <v>844716.5965149167</v>
       </c>
       <c r="D131" s="6" t="n">
-        <v>824441.9861349808</v>
+        <v>824441.9861349809</v>
       </c>
       <c r="E131" s="6" t="n">
         <v>825491.5320733978</v>
@@ -5142,16 +5164,16 @@
         <v>1</v>
       </c>
       <c r="B132" s="7" t="n">
-        <v>749354.3278026374</v>
+        <v>749354.3278026375</v>
       </c>
       <c r="C132" s="7" t="n">
         <v>797082.4788724037</v>
       </c>
       <c r="D132" s="7" t="n">
-        <v>755910.4055846768</v>
+        <v>755910.4055846769</v>
       </c>
       <c r="E132" s="7" t="n">
-        <v>756036.7141654211</v>
+        <v>756036.7141654212</v>
       </c>
       <c r="F132" s="8" t="n"/>
     </row>
@@ -5163,7 +5185,7 @@
         <v>686613.3653028569</v>
       </c>
       <c r="C133" s="6" t="n">
-        <v>719919.150540015</v>
+        <v>719919.1505400151</v>
       </c>
       <c r="D133" s="6" t="n">
         <v>691007.5050956833</v>
@@ -5538,16 +5560,16 @@
         <v>0.05</v>
       </c>
       <c r="B160" s="6" t="n">
-        <v>7.682050698262174</v>
+        <v>5.650267199496739</v>
       </c>
       <c r="C160" s="6" t="n">
-        <v>65.78858370281523</v>
+        <v>57.18830979574705</v>
       </c>
       <c r="D160" s="6" t="n">
-        <v>2081.548187398526</v>
+        <v>2184.058027800347</v>
       </c>
       <c r="E160" s="6" t="n">
-        <v>15.69642789848149</v>
+        <v>14.46445210085949</v>
       </c>
     </row>
     <row r="161">
@@ -5555,16 +5577,16 @@
         <v>0.1</v>
       </c>
       <c r="B161" s="7" t="n">
-        <v>7.704395500652026</v>
+        <v>7.316266800044104</v>
       </c>
       <c r="C161" s="7" t="n">
-        <v>22.01719390077051</v>
+        <v>20.57438839913812</v>
       </c>
       <c r="D161" s="7" t="n">
-        <v>551.7031286003185</v>
+        <v>553.0384970997111</v>
       </c>
       <c r="E161" s="7" t="n">
-        <v>9.770100601017475</v>
+        <v>9.338120498869102</v>
       </c>
     </row>
     <row r="162">
@@ -5572,16 +5594,16 @@
         <v>0.5</v>
       </c>
       <c r="B162" s="6" t="n">
-        <v>3.476132399810012</v>
+        <v>3.675169599882793</v>
       </c>
       <c r="C162" s="6" t="n">
-        <v>3.870809999876656</v>
+        <v>4.180422900128178</v>
       </c>
       <c r="D162" s="6" t="n">
-        <v>23.81353889999446</v>
+        <v>41.60657289996743</v>
       </c>
       <c r="E162" s="6" t="n">
-        <v>3.540848599455785</v>
+        <v>3.725207199691795</v>
       </c>
     </row>
     <row r="163">
@@ -5589,16 +5611,16 @@
         <v>1</v>
       </c>
       <c r="B163" s="7" t="n">
-        <v>3.420683500065934</v>
+        <v>3.564584199979436</v>
       </c>
       <c r="C163" s="7" t="n">
-        <v>3.505551300069783</v>
+        <v>3.649123599985614</v>
       </c>
       <c r="D163" s="7" t="n">
-        <v>9.770413400023244</v>
+        <v>11.43315789994085</v>
       </c>
       <c r="E163" s="7" t="n">
-        <v>3.450090300117154</v>
+        <v>3.578195900015999</v>
       </c>
     </row>
     <row r="164">
@@ -5606,16 +5628,16 @@
         <v>2</v>
       </c>
       <c r="B164" s="6" t="n">
-        <v>3.38530260004336</v>
+        <v>3.531848100072239</v>
       </c>
       <c r="C164" s="6" t="n">
-        <v>3.40095369995106</v>
+        <v>3.551406599988695</v>
       </c>
       <c r="D164" s="6" t="n">
-        <v>4.131573199992999</v>
+        <v>4.574743799981661</v>
       </c>
       <c r="E164" s="6" t="n">
-        <v>3.387840599985793</v>
+        <v>3.534459000104107</v>
       </c>
     </row>
     <row r="165">
@@ -5623,16 +5645,16 @@
         <v>5</v>
       </c>
       <c r="B165" s="7" t="n">
-        <v>3.48771019995911</v>
+        <v>3.631156700022984</v>
       </c>
       <c r="C165" s="7" t="n">
-        <v>3.490616400027648</v>
+        <v>3.63420790003147</v>
       </c>
       <c r="D165" s="7" t="n">
-        <v>3.566732800041791</v>
+        <v>3.71802899998147</v>
       </c>
       <c r="E165" s="7" t="n">
-        <v>3.4883198000025</v>
+        <v>3.631619499996305</v>
       </c>
     </row>
     <row r="166">
@@ -5640,16 +5662,16 @@
         <v>10</v>
       </c>
       <c r="B166" s="6" t="n">
-        <v>3.56765969999833</v>
+        <v>3.760585299984086</v>
       </c>
       <c r="C166" s="6" t="n">
-        <v>3.568274399964139</v>
+        <v>3.761388599989004</v>
       </c>
       <c r="D166" s="6" t="n">
-        <v>3.588710499985609</v>
+        <v>3.782736199966166</v>
       </c>
       <c r="E166" s="6" t="n">
-        <v>3.567948899988551</v>
+        <v>3.760792399989441</v>
       </c>
     </row>
     <row r="167">
@@ -5657,16 +5679,16 @@
         <v>20</v>
       </c>
       <c r="B167" s="7" t="n">
-        <v>3.733965899969917</v>
+        <v>3.933920799987391</v>
       </c>
       <c r="C167" s="7" t="n">
-        <v>3.734140799962915</v>
+        <v>3.934117900033016</v>
       </c>
       <c r="D167" s="7" t="n">
-        <v>3.740086499950849</v>
+        <v>3.940273899992462</v>
       </c>
       <c r="E167" s="7" t="n">
-        <v>3.734080499911215</v>
+        <v>3.934063399967272</v>
       </c>
     </row>
     <row r="168">
@@ -5674,16 +5696,16 @@
         <v>50</v>
       </c>
       <c r="B168" s="6" t="n">
-        <v>5.181382800044958</v>
+        <v>5.325104300049134</v>
       </c>
       <c r="C168" s="6" t="n">
-        <v>5.18144640000537</v>
+        <v>5.325089799996931</v>
       </c>
       <c r="D168" s="6" t="n">
-        <v>5.183720800036099</v>
+        <v>5.327653599961195</v>
       </c>
       <c r="E168" s="6" t="n">
-        <v>5.181476000056136</v>
+        <v>5.325148199975956</v>
       </c>
     </row>
     <row r="171" ht="20" customHeight="1">
@@ -5737,25 +5759,25 @@
     </row>
     <row r="173">
       <c r="A173" s="6" t="n">
-        <v>7.682050698262174</v>
+        <v>5.650267199496739</v>
       </c>
       <c r="B173" s="6" t="n">
         <v>0.0004732261803341386</v>
       </c>
       <c r="C173" s="6" t="n">
-        <v>65.78858370281523</v>
+        <v>57.18830979574705</v>
       </c>
       <c r="D173" s="6" t="n">
         <v>0.0001210799605146639</v>
       </c>
       <c r="E173" s="6" t="n">
-        <v>2081.548187398526</v>
+        <v>2184.058027800347</v>
       </c>
       <c r="F173" s="6" t="n">
         <v>0.0004261445917168604</v>
       </c>
       <c r="G173" s="6" t="n">
-        <v>15.69642789848149</v>
+        <v>14.46445210085949</v>
       </c>
       <c r="H173" s="6" t="n">
         <v>0.0004029868368585799</v>

</xml_diff>